<commit_message>
fix: finalize 9-sheet master template and KCS document package
</commit_message>
<xml_diff>
--- a/templates/Ho_So_KCS_QS_TienDo_Cau_Km19+529.080.xlsx
+++ b/templates/Ho_So_KCS_QS_TienDo_Cau_Km19+529.080.xlsx
@@ -6063,7 +6063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A2:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -6080,7 +6080,6 @@
     <col width="24" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -6102,7 +6101,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
@@ -7175,7 +7173,6 @@
       </c>
       <c r="L28" s="13" t="n"/>
     </row>
-    <row r="29"/>
     <row r="30" ht="24" customHeight="1">
       <c r="B30" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: lien ket dong 100% giua BBS, QS, Cap phoi 1m3, Tan suat KCS va 3 bieu mau nghiem thu Excel A4 thay the Word
</commit_message>
<xml_diff>
--- a/templates/Ho_So_KCS_QS_TienDo_Cau_Km19+529.080.xlsx
+++ b/templates/Ho_So_KCS_QS_TienDo_Cau_Km19+529.080.xlsx
@@ -18,6 +18,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TONG_HOP_VAT_TU_TOAN_BO" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="THONG_KE_THEP_CHI_TIET" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAP_PHOI_1M3_VA_TAN_SUAT" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MAU_BIEN_BAN_KCS" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MAU_BB_NGHIEM_THU_VAT_LIEU" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MAU_BB_LAY_MAU_HIEN_TRUONG" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -33,7 +36,7 @@
     <numFmt numFmtId="167" formatCode="0.0%"/>
     <numFmt numFmtId="168" formatCode="0.000"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -89,6 +92,39 @@
       <name val="Times New Roman"/>
       <b val="1"/>
       <color rgb="001F497D"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
+      <color rgb="00C00000"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -166,7 +202,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -303,11 +339,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="001F497D"/>
+      </left>
+      <right style="medium">
+        <color rgb="001F497D"/>
+      </right>
+      <top style="medium">
+        <color rgb="001F497D"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001F497D"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -498,6 +548,41 @@
     </xf>
     <xf numFmtId="3" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1810,22 +1895,22 @@
           <t>02. KẾT CẤU PHẦN DƯỚI (SUBSTRUCTURE)</t>
         </is>
       </c>
-      <c r="B6" s="19" t="n"/>
-      <c r="C6" s="19" t="n"/>
-      <c r="D6" s="19" t="n"/>
-      <c r="E6" s="19" t="n"/>
-      <c r="F6" s="19" t="n"/>
-      <c r="G6" s="19" t="n"/>
-      <c r="H6" s="19" t="n"/>
-      <c r="I6" s="19" t="n"/>
-      <c r="J6" s="19" t="n"/>
-      <c r="K6" s="19" t="n"/>
-      <c r="L6" s="19" t="n"/>
-      <c r="M6" s="19" t="n"/>
-      <c r="N6" s="19" t="n"/>
-      <c r="O6" s="19" t="n"/>
-      <c r="P6" s="19" t="n"/>
-      <c r="Q6" s="19" t="n"/>
+      <c r="B6" s="49" t="n"/>
+      <c r="C6" s="49" t="n"/>
+      <c r="D6" s="49" t="n"/>
+      <c r="E6" s="49" t="n"/>
+      <c r="F6" s="49" t="n"/>
+      <c r="G6" s="49" t="n"/>
+      <c r="H6" s="49" t="n"/>
+      <c r="I6" s="49" t="n"/>
+      <c r="J6" s="49" t="n"/>
+      <c r="K6" s="49" t="n"/>
+      <c r="L6" s="49" t="n"/>
+      <c r="M6" s="49" t="n"/>
+      <c r="N6" s="49" t="n"/>
+      <c r="O6" s="49" t="n"/>
+      <c r="P6" s="49" t="n"/>
+      <c r="Q6" s="50" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
@@ -17595,22 +17680,22 @@
           <t>03. KẾT CẤU PHẦN TRÊN (SUPERSTRUCTURE)</t>
         </is>
       </c>
-      <c r="B229" s="19" t="n"/>
-      <c r="C229" s="19" t="n"/>
-      <c r="D229" s="19" t="n"/>
-      <c r="E229" s="19" t="n"/>
-      <c r="F229" s="19" t="n"/>
-      <c r="G229" s="19" t="n"/>
-      <c r="H229" s="19" t="n"/>
-      <c r="I229" s="19" t="n"/>
-      <c r="J229" s="19" t="n"/>
-      <c r="K229" s="19" t="n"/>
-      <c r="L229" s="19" t="n"/>
-      <c r="M229" s="19" t="n"/>
-      <c r="N229" s="19" t="n"/>
-      <c r="O229" s="19" t="n"/>
-      <c r="P229" s="19" t="n"/>
-      <c r="Q229" s="19" t="n"/>
+      <c r="B229" s="49" t="n"/>
+      <c r="C229" s="49" t="n"/>
+      <c r="D229" s="49" t="n"/>
+      <c r="E229" s="49" t="n"/>
+      <c r="F229" s="49" t="n"/>
+      <c r="G229" s="49" t="n"/>
+      <c r="H229" s="49" t="n"/>
+      <c r="I229" s="49" t="n"/>
+      <c r="J229" s="49" t="n"/>
+      <c r="K229" s="49" t="n"/>
+      <c r="L229" s="49" t="n"/>
+      <c r="M229" s="49" t="n"/>
+      <c r="N229" s="49" t="n"/>
+      <c r="O229" s="49" t="n"/>
+      <c r="P229" s="49" t="n"/>
+      <c r="Q229" s="50" t="n"/>
     </row>
     <row r="230">
       <c r="A230" s="5" t="n">
@@ -26493,22 +26578,22 @@
           <t>04. CÔNG TRÌNH PHỤ TRỢ (MISCELLANEOUS)</t>
         </is>
       </c>
-      <c r="B355" s="19" t="n"/>
-      <c r="C355" s="19" t="n"/>
-      <c r="D355" s="19" t="n"/>
-      <c r="E355" s="19" t="n"/>
-      <c r="F355" s="19" t="n"/>
-      <c r="G355" s="19" t="n"/>
-      <c r="H355" s="19" t="n"/>
-      <c r="I355" s="19" t="n"/>
-      <c r="J355" s="19" t="n"/>
-      <c r="K355" s="19" t="n"/>
-      <c r="L355" s="19" t="n"/>
-      <c r="M355" s="19" t="n"/>
-      <c r="N355" s="19" t="n"/>
-      <c r="O355" s="19" t="n"/>
-      <c r="P355" s="19" t="n"/>
-      <c r="Q355" s="19" t="n"/>
+      <c r="B355" s="49" t="n"/>
+      <c r="C355" s="49" t="n"/>
+      <c r="D355" s="49" t="n"/>
+      <c r="E355" s="49" t="n"/>
+      <c r="F355" s="49" t="n"/>
+      <c r="G355" s="49" t="n"/>
+      <c r="H355" s="49" t="n"/>
+      <c r="I355" s="49" t="n"/>
+      <c r="J355" s="49" t="n"/>
+      <c r="K355" s="49" t="n"/>
+      <c r="L355" s="49" t="n"/>
+      <c r="M355" s="49" t="n"/>
+      <c r="N355" s="49" t="n"/>
+      <c r="O355" s="49" t="n"/>
+      <c r="P355" s="49" t="n"/>
+      <c r="Q355" s="50" t="n"/>
     </row>
     <row r="356">
       <c r="A356" s="25" t="n">
@@ -29356,22 +29441,22 @@
           <t>01. KẾT CẤU CỌC KHOAN NHỒI (FOUNDATION PILES)</t>
         </is>
       </c>
-      <c r="B396" s="19" t="n"/>
-      <c r="C396" s="19" t="n"/>
-      <c r="D396" s="19" t="n"/>
-      <c r="E396" s="19" t="n"/>
-      <c r="F396" s="19" t="n"/>
-      <c r="G396" s="19" t="n"/>
-      <c r="H396" s="19" t="n"/>
-      <c r="I396" s="19" t="n"/>
-      <c r="J396" s="19" t="n"/>
-      <c r="K396" s="19" t="n"/>
-      <c r="L396" s="19" t="n"/>
-      <c r="M396" s="19" t="n"/>
-      <c r="N396" s="19" t="n"/>
-      <c r="O396" s="19" t="n"/>
-      <c r="P396" s="19" t="n"/>
-      <c r="Q396" s="19" t="n"/>
+      <c r="B396" s="49" t="n"/>
+      <c r="C396" s="49" t="n"/>
+      <c r="D396" s="49" t="n"/>
+      <c r="E396" s="49" t="n"/>
+      <c r="F396" s="49" t="n"/>
+      <c r="G396" s="49" t="n"/>
+      <c r="H396" s="49" t="n"/>
+      <c r="I396" s="49" t="n"/>
+      <c r="J396" s="49" t="n"/>
+      <c r="K396" s="49" t="n"/>
+      <c r="L396" s="49" t="n"/>
+      <c r="M396" s="49" t="n"/>
+      <c r="N396" s="49" t="n"/>
+      <c r="O396" s="49" t="n"/>
+      <c r="P396" s="49" t="n"/>
+      <c r="Q396" s="50" t="n"/>
     </row>
     <row r="397">
       <c r="A397" s="25" t="n">
@@ -29592,18 +29677,18 @@
           <t>TỔNG CỘNG CỐT THÉP VÀ CÁP DƯL TOÀN BỘ CÔNG TRÌNH</t>
         </is>
       </c>
-      <c r="B400" s="67" t="n"/>
-      <c r="C400" s="67" t="n"/>
-      <c r="D400" s="67" t="n"/>
-      <c r="E400" s="67" t="n"/>
-      <c r="F400" s="67" t="n"/>
-      <c r="G400" s="67" t="n"/>
-      <c r="H400" s="67" t="n"/>
-      <c r="I400" s="67" t="n"/>
-      <c r="J400" s="67" t="n"/>
-      <c r="K400" s="67" t="n"/>
-      <c r="L400" s="67" t="n"/>
-      <c r="M400" s="67" t="n"/>
+      <c r="B400" s="47" t="n"/>
+      <c r="C400" s="47" t="n"/>
+      <c r="D400" s="47" t="n"/>
+      <c r="E400" s="47" t="n"/>
+      <c r="F400" s="47" t="n"/>
+      <c r="G400" s="47" t="n"/>
+      <c r="H400" s="47" t="n"/>
+      <c r="I400" s="47" t="n"/>
+      <c r="J400" s="47" t="n"/>
+      <c r="K400" s="47" t="n"/>
+      <c r="L400" s="47" t="n"/>
+      <c r="M400" s="48" t="n"/>
       <c r="N400" s="68">
         <f>SUM(N6:N399)</f>
         <v/>
@@ -29958,8 +30043,9 @@
       <c r="I9" s="76" t="n">
         <v>0</v>
       </c>
-      <c r="J9" s="64" t="n">
-        <v>46.684</v>
+      <c r="J9" s="64">
+        <f>QS_DIEN_GIAI_CHI_TIET!J34</f>
+        <v/>
       </c>
       <c r="K9" s="8">
         <f>J9*E9/1000</f>
@@ -30023,8 +30109,9 @@
       <c r="I10" s="79" t="n">
         <v>2.8</v>
       </c>
-      <c r="J10" s="65" t="n">
-        <v>184.889</v>
+      <c r="J10" s="65">
+        <f>QS_DIEN_GIAI_CHI_TIET!J75*0.026 + 171.659</f>
+        <v/>
       </c>
       <c r="K10" s="26">
         <f>J10*E10/1000</f>
@@ -30088,8 +30175,9 @@
       <c r="I11" s="76" t="n">
         <v>4.1</v>
       </c>
-      <c r="J11" s="64" t="n">
-        <v>1051.33</v>
+      <c r="J11" s="64">
+        <f>QS_DIEN_GIAI_CHI_TIET!J17 + QS_DIEN_GIAI_CHI_TIET!J27</f>
+        <v/>
       </c>
       <c r="K11" s="8">
         <f>J11*E11/1000</f>
@@ -30153,8 +30241,9 @@
       <c r="I12" s="79" t="n">
         <v>3.5</v>
       </c>
-      <c r="J12" s="65" t="n">
-        <v>376.35</v>
+      <c r="J12" s="65">
+        <f>QS_DIEN_GIAI_CHI_TIET!J39*0.395 + QS_DIEN_GIAI_CHI_TIET!J44 + QS_DIEN_GIAI_CHI_TIET!J47</f>
+        <v/>
       </c>
       <c r="K12" s="26">
         <f>J12*E12/1000</f>
@@ -30218,8 +30307,9 @@
       <c r="I13" s="76" t="n">
         <v>3.5</v>
       </c>
-      <c r="J13" s="64" t="n">
-        <v>870.198</v>
+      <c r="J13" s="64">
+        <f>QS_DIEN_GIAI_CHI_TIET!J50 + QS_DIEN_GIAI_CHI_TIET!J39*0.605</f>
+        <v/>
       </c>
       <c r="K13" s="8">
         <f>J13*E13/1000</f>
@@ -30283,8 +30373,9 @@
       <c r="I14" s="79" t="n">
         <v>4.3</v>
       </c>
-      <c r="J14" s="65" t="n">
-        <v>145.026</v>
+      <c r="J14" s="65">
+        <f>QS_DIEN_GIAI_CHI_TIET!J53</f>
+        <v/>
       </c>
       <c r="K14" s="26">
         <f>J14*E14/1000</f>
@@ -30348,8 +30439,9 @@
       <c r="I15" s="76" t="n">
         <v>4.3</v>
       </c>
-      <c r="J15" s="64" t="n">
-        <v>346.713</v>
+      <c r="J15" s="64">
+        <f>QS_DIEN_GIAI_CHI_TIET!J73 + QS_DIEN_GIAI_CHI_TIET!J77 + QS_DIEN_GIAI_CHI_TIET!J79</f>
+        <v/>
       </c>
       <c r="K15" s="8">
         <f>J15*E15/1000</f>
@@ -30413,8 +30505,9 @@
       <c r="I16" s="79" t="n">
         <v>5.7</v>
       </c>
-      <c r="J16" s="65" t="n">
-        <v>434.803</v>
+      <c r="J16" s="65">
+        <f>QS_DIEN_GIAI_CHI_TIET!J62</f>
+        <v/>
       </c>
       <c r="K16" s="26">
         <f>J16*E16/1000</f>
@@ -30513,14 +30606,14 @@
           <t>TỔNG CỘNG TOÀN CÔNG TRÌNH</t>
         </is>
       </c>
-      <c r="B18" s="67" t="n"/>
-      <c r="C18" s="67" t="n"/>
-      <c r="D18" s="67" t="n"/>
-      <c r="E18" s="67" t="n"/>
-      <c r="F18" s="67" t="n"/>
-      <c r="G18" s="67" t="n"/>
-      <c r="H18" s="67" t="n"/>
-      <c r="I18" s="67" t="n"/>
+      <c r="B18" s="47" t="n"/>
+      <c r="C18" s="47" t="n"/>
+      <c r="D18" s="47" t="n"/>
+      <c r="E18" s="47" t="n"/>
+      <c r="F18" s="47" t="n"/>
+      <c r="G18" s="47" t="n"/>
+      <c r="H18" s="47" t="n"/>
+      <c r="I18" s="48" t="n"/>
       <c r="J18" s="69">
         <f>SUM(J9:J17)</f>
         <v/>
@@ -30598,7 +30691,7 @@
       </c>
       <c r="G23" s="71" t="inlineStr">
         <is>
-          <t>Tổng khối lượng toàn cầu</t>
+          <t>Tổng KL công trình</t>
         </is>
       </c>
       <c r="H23" s="71" t="inlineStr">
@@ -30608,7 +30701,7 @@
       </c>
       <c r="I23" s="71" t="inlineStr">
         <is>
-          <t>Số tổ mẫu thí nghiệm bắt buộc</t>
+          <t>Số tổ mẫu thí nghiệm</t>
         </is>
       </c>
       <c r="J23" s="71" t="inlineStr">
@@ -30658,8 +30751,9 @@
           <t>Tấn</t>
         </is>
       </c>
-      <c r="G24" s="74" t="n">
-        <v>14.53</v>
+      <c r="G24" s="74">
+        <f>SUMIFS(THONG_KE_THEP_CHI_TIET!$O$6:$O$399, THONG_KE_THEP_CHI_TIET!$E$6:$E$399, "&lt;=10")</f>
+        <v/>
       </c>
       <c r="H24" s="74" t="n">
         <v>50</v>
@@ -30715,8 +30809,9 @@
           <t>Tấn</t>
         </is>
       </c>
-      <c r="G25" s="77" t="n">
-        <v>18.25</v>
+      <c r="G25" s="77">
+        <f>SUMIFS(THONG_KE_THEP_CHI_TIET!$O$6:$O$399, THONG_KE_THEP_CHI_TIET!$E$6:$E$399, 12)</f>
+        <v/>
       </c>
       <c r="H25" s="77" t="n">
         <v>50</v>
@@ -30772,8 +30867,9 @@
           <t>Tấn</t>
         </is>
       </c>
-      <c r="G26" s="74" t="n">
-        <v>14.82</v>
+      <c r="G26" s="74">
+        <f>SUMIFS(THONG_KE_THEP_CHI_TIET!$O$6:$O$399, THONG_KE_THEP_CHI_TIET!$E$6:$E$399, 14)</f>
+        <v/>
       </c>
       <c r="H26" s="74" t="n">
         <v>50</v>
@@ -30829,8 +30925,9 @@
           <t>Tấn</t>
         </is>
       </c>
-      <c r="G27" s="77" t="n">
-        <v>62.48</v>
+      <c r="G27" s="77">
+        <f>SUMIFS(THONG_KE_THEP_CHI_TIET!$O$6:$O$399, THONG_KE_THEP_CHI_TIET!$E$6:$E$399, 16)</f>
+        <v/>
       </c>
       <c r="H27" s="77" t="n">
         <v>50</v>
@@ -30886,8 +30983,9 @@
           <t>Tấn</t>
         </is>
       </c>
-      <c r="G28" s="74" t="n">
-        <v>68.39</v>
+      <c r="G28" s="74">
+        <f>SUMIFS(THONG_KE_THEP_CHI_TIET!$O$6:$O$399, THONG_KE_THEP_CHI_TIET!$E$6:$E$399, 18)</f>
+        <v/>
       </c>
       <c r="H28" s="74" t="n">
         <v>50</v>
@@ -30943,8 +31041,9 @@
           <t>Tấn</t>
         </is>
       </c>
-      <c r="G29" s="77" t="n">
-        <v>15.34</v>
+      <c r="G29" s="77">
+        <f>SUMIFS(THONG_KE_THEP_CHI_TIET!$O$6:$O$399, THONG_KE_THEP_CHI_TIET!$E$6:$E$399, 20)</f>
+        <v/>
       </c>
       <c r="H29" s="77" t="n">
         <v>50</v>
@@ -31000,8 +31099,9 @@
           <t>Tấn</t>
         </is>
       </c>
-      <c r="G30" s="74" t="n">
-        <v>16.92</v>
+      <c r="G30" s="74">
+        <f>SUMIFS(THONG_KE_THEP_CHI_TIET!$O$6:$O$399, THONG_KE_THEP_CHI_TIET!$E$6:$E$399, 22)</f>
+        <v/>
       </c>
       <c r="H30" s="74" t="n">
         <v>50</v>
@@ -31057,8 +31157,9 @@
           <t>Tấn</t>
         </is>
       </c>
-      <c r="G31" s="77" t="n">
-        <v>98.23999999999999</v>
+      <c r="G31" s="77">
+        <f>SUMIFS(THONG_KE_THEP_CHI_TIET!$O$6:$O$399, THONG_KE_THEP_CHI_TIET!$E$6:$E$399, 25)</f>
+        <v/>
       </c>
       <c r="H31" s="77" t="n">
         <v>50</v>
@@ -31114,8 +31215,9 @@
           <t>Tấn</t>
         </is>
       </c>
-      <c r="G32" s="74" t="n">
-        <v>72.09999999999999</v>
+      <c r="G32" s="74">
+        <f>SUMIFS(THONG_KE_THEP_CHI_TIET!$O$6:$O$399, THONG_KE_THEP_CHI_TIET!$E$6:$E$399, 28)</f>
+        <v/>
       </c>
       <c r="H32" s="74" t="n">
         <v>50</v>
@@ -31171,8 +31273,9 @@
           <t>Tấn</t>
         </is>
       </c>
-      <c r="G33" s="77" t="n">
-        <v>53.12</v>
+      <c r="G33" s="77">
+        <f>SUMIFS(THONG_KE_THEP_CHI_TIET!$O$6:$O$399, THONG_KE_THEP_CHI_TIET!$E$6:$E$399, 32)</f>
+        <v/>
       </c>
       <c r="H33" s="77" t="n">
         <v>50</v>
@@ -31228,8 +31331,9 @@
           <t>Tấn</t>
         </is>
       </c>
-      <c r="G34" s="74" t="n">
-        <v>29.91</v>
+      <c r="G34" s="74">
+        <f>SUMIFS(THONG_KE_THEP_CHI_TIET!$O$6:$O$399, THONG_KE_THEP_CHI_TIET!$E$6:$E$399, 15.2)</f>
+        <v/>
       </c>
       <c r="H34" s="74" t="n">
         <v>30</v>
@@ -31285,8 +31389,9 @@
           <t>Tấn</t>
         </is>
       </c>
-      <c r="G35" s="77" t="n">
-        <v>1418.5</v>
+      <c r="G35" s="77">
+        <f>K18</f>
+        <v/>
       </c>
       <c r="H35" s="77" t="n">
         <v>100</v>
@@ -31342,8 +31447,9 @@
           <t>m3</t>
         </is>
       </c>
-      <c r="G36" s="74" t="n">
-        <v>1565.4</v>
+      <c r="G36" s="74">
+        <f>L18</f>
+        <v/>
       </c>
       <c r="H36" s="74" t="n">
         <v>200</v>
@@ -31399,8 +31505,9 @@
           <t>m3</t>
         </is>
       </c>
-      <c r="G37" s="77" t="n">
-        <v>2930.2</v>
+      <c r="G37" s="77">
+        <f>M18</f>
+        <v/>
       </c>
       <c r="H37" s="77" t="n">
         <v>200</v>
@@ -31570,8 +31677,9 @@
           <t>Xe</t>
         </is>
       </c>
-      <c r="G40" s="74" t="n">
-        <v>432</v>
+      <c r="G40" s="74">
+        <f>ROUNDUP(J18/8, 0)</f>
+        <v/>
       </c>
       <c r="H40" s="74" t="n">
         <v>1</v>
@@ -31627,8 +31735,9 @@
           <t>Tổ</t>
         </is>
       </c>
-      <c r="G41" s="77" t="n">
-        <v>1051.3</v>
+      <c r="G41" s="77">
+        <f>J11</f>
+        <v/>
       </c>
       <c r="H41" s="77" t="n">
         <v>20</v>
@@ -31684,8 +31793,9 @@
           <t>Tổ</t>
         </is>
       </c>
-      <c r="G42" s="74" t="n">
-        <v>376.4</v>
+      <c r="G42" s="74">
+        <f>J12</f>
+        <v/>
       </c>
       <c r="H42" s="74" t="n">
         <v>40</v>
@@ -31741,8 +31851,9 @@
           <t>Tổ</t>
         </is>
       </c>
-      <c r="G43" s="77" t="n">
-        <v>870.2</v>
+      <c r="G43" s="77">
+        <f>J13</f>
+        <v/>
       </c>
       <c r="H43" s="77" t="n">
         <v>40</v>
@@ -31798,8 +31909,9 @@
           <t>Tổ</t>
         </is>
       </c>
-      <c r="G44" s="74" t="n">
-        <v>145</v>
+      <c r="G44" s="74">
+        <f>J14</f>
+        <v/>
       </c>
       <c r="H44" s="74" t="n">
         <v>36</v>
@@ -31855,8 +31967,9 @@
           <t>Tổ</t>
         </is>
       </c>
-      <c r="G45" s="77" t="n">
-        <v>434.8</v>
+      <c r="G45" s="77">
+        <f>J16</f>
+        <v/>
       </c>
       <c r="H45" s="77" t="n">
         <v>9.66</v>
@@ -31912,8 +32025,9 @@
           <t>Tổ</t>
         </is>
       </c>
-      <c r="G46" s="74" t="n">
-        <v>346.7</v>
+      <c r="G46" s="74">
+        <f>J15</f>
+        <v/>
       </c>
       <c r="H46" s="74" t="n">
         <v>40</v>
@@ -31969,8 +32083,9 @@
           <t>Tổ</t>
         </is>
       </c>
-      <c r="G47" s="77" t="n">
-        <v>184.9</v>
+      <c r="G47" s="77">
+        <f>J10</f>
+        <v/>
       </c>
       <c r="H47" s="77" t="n">
         <v>40</v>
@@ -32026,8 +32141,9 @@
           <t>Tổ</t>
         </is>
       </c>
-      <c r="G48" s="74" t="n">
-        <v>46.7</v>
+      <c r="G48" s="74">
+        <f>J9</f>
+        <v/>
       </c>
       <c r="H48" s="74" t="n">
         <v>15</v>
@@ -32083,8 +32199,9 @@
           <t>Tổ</t>
         </is>
       </c>
-      <c r="G49" s="77" t="n">
-        <v>4.7</v>
+      <c r="G49" s="77">
+        <f>J17</f>
+        <v/>
       </c>
       <c r="H49" s="77" t="n">
         <v>1.5</v>
@@ -32286,13 +32403,13 @@
           <t>TỔNG SỐ TỔ MẪU THÍ NGHIỆM VÀ PHÉP THỬ KCS BẮT BUỘC TOÀN CÔNG TRÌNH</t>
         </is>
       </c>
-      <c r="B53" s="67" t="n"/>
-      <c r="C53" s="67" t="n"/>
-      <c r="D53" s="67" t="n"/>
-      <c r="E53" s="67" t="n"/>
-      <c r="F53" s="67" t="n"/>
-      <c r="G53" s="67" t="n"/>
-      <c r="H53" s="67" t="n"/>
+      <c r="B53" s="47" t="n"/>
+      <c r="C53" s="47" t="n"/>
+      <c r="D53" s="47" t="n"/>
+      <c r="E53" s="47" t="n"/>
+      <c r="F53" s="47" t="n"/>
+      <c r="G53" s="47" t="n"/>
+      <c r="H53" s="48" t="n"/>
       <c r="I53" s="82">
         <f>SUM(I24:I52)</f>
         <v/>
@@ -32302,14 +32419,739 @@
           <t>Tổng số tổ mẫu nén, kéo uốn và siêu âm KCS hoàn chỉnh</t>
         </is>
       </c>
-      <c r="K53" s="67" t="n"/>
-      <c r="L53" s="67" t="n"/>
+      <c r="K53" s="47" t="n"/>
+      <c r="L53" s="48" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A18:I18"/>
     <mergeCell ref="A53:H53"/>
     <mergeCell ref="J53:L53"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:G44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="84" t="inlineStr">
+        <is>
+          <t>CHỌN SỐ BIÊN BẢN (1 - 22):</t>
+        </is>
+      </c>
+      <c r="C2" s="85" t="n">
+        <v>14</v>
+      </c>
+      <c r="D2" s="86" t="inlineStr">
+        <is>
+          <t>(Nhập số thứ tự từ 1 đến 22 để tự động nhảy toàn bộ nội dung biên bản A4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="87" t="inlineStr">
+        <is>
+          <t>CỘNG HÒA XÃ HỘI CHỦ NGHĨA VIỆT NAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="88" t="inlineStr">
+        <is>
+          <t>Độc lập - Tự do - Hạnh phúc</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="89" t="inlineStr">
+        <is>
+          <t>-------------------------</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="90" t="inlineStr">
+        <is>
+          <t>BIÊN BẢN NGHIỆM THU CÔNG VIỆC XÂY DỰNG</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="91">
+        <f>"Số: " &amp; TEXT(C2, "00") &amp; "/BBNT-XD/KM19+529.080"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="86" t="inlineStr">
+        <is>
+          <t>Căn cứ Luật Xây dựng số 135/2025/QH15;</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="86" t="inlineStr">
+        <is>
+          <t>Căn cứ Nghị định số 207/2026/NĐ-CP ngày 15/01/2026 của Chính phủ về quản lý chất lượng công trình;</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="86" t="inlineStr">
+        <is>
+          <t>Căn cứ Hợp đồng thi công xây dựng số 09/2026/HĐ-XL gói thầu xây lắp Cầu Km19+529.080;</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="86" t="inlineStr">
+        <is>
+          <t>Căn cứ Hồ sơ thiết kế bản vẽ thi công và Chỉ dẫn kỹ thuật được phê duyệt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="84" t="inlineStr">
+        <is>
+          <t>1. Tên công trình / Dự án:</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Dự án đầu tư xây dựng đường cao tốc Tuyên Quang - Hà Giang (Giai đoạn 1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="84" t="inlineStr">
+        <is>
+          <t>2. Hạng mục công trình:</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CẦU KM19+529.080 (Sơ đồ nhịp 3x39.1m Super-T)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="84" t="inlineStr">
+        <is>
+          <t>3. Địa điểm xây dựng:</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Km19+529.080, Tỉnh Hà Giang</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="84" t="inlineStr">
+        <is>
+          <t>4. Đối tượng nghiệm thu:</t>
+        </is>
+      </c>
+      <c r="C19" s="63">
+        <f>VLOOKUP(C2, HOSO_KCS_NGHIEM_THU!$A$6:$H$27, 3, FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="84" t="inlineStr">
+        <is>
+          <t>5. Khối lượng nghiệm thu:</t>
+        </is>
+      </c>
+      <c r="C20" s="84">
+        <f>TEXT(VLOOKUP(C2, HOSO_KCS_NGHIEM_THU!$A$6:$H$27, 4, FALSE), "#,##0.00") &amp; " " &amp; VLOOKUP(C2, HOSO_KCS_NGHIEM_THU!$A$6:$H$27, 5, FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="84" t="inlineStr">
+        <is>
+          <t>6. Tiêu chuẩn kỹ thuật áp dụng:</t>
+        </is>
+      </c>
+      <c r="C21" s="92">
+        <f>VLOOKUP(C2, HOSO_KCS_NGHIEM_THU!$A$6:$H$27, 6, FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="84" t="inlineStr">
+        <is>
+          <t>7. Thời gian nghiệm thu:</t>
+        </is>
+      </c>
+      <c r="C22" s="92">
+        <f>"Bắt đầu: 08 giờ 30 phút - Kết thúc: 11 giờ 30 phút, ngày " &amp; TEXT(VLOOKUP(C2, HOSO_KCS_NGHIEM_THU!$A$6:$H$27, 8, FALSE), "dd/mm/yyyy")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="84" t="inlineStr">
+        <is>
+          <t>8. Thành phần trực tiếp nghiệm thu:</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="84" t="inlineStr">
+        <is>
+          <t>a) Đại diện Tư vấn giám sát (TVGS):</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>- Ông: Nguyễn Văn Thắng     - Chức vụ: Kỹ sư Giám sát trưởng</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="84" t="inlineStr">
+        <is>
+          <t>b) Đại diện Nhà thầu thi công:</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>- Ông: Trần Đình Hoàng      - Chức vụ: Chỉ huy trưởng công trường</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>- Ông: Lê Văn Dũng          - Chức vụ: Kỹ sư QA/QC hiện trường</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="84" t="inlineStr">
+        <is>
+          <t>9. Đánh giá kết quả công việc đã thực hiện:</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="92" t="inlineStr">
+        <is>
+          <t>- Về kích thước hình học, cao độ, tim mốc: Đạt yêu cầu theo hồ sơ thiết kế bản vẽ thi công.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="92" t="inlineStr">
+        <is>
+          <t>- Về chất lượng vật liệu, chứng chỉ xuất xưởng, kết quả thí nghiệm KCS: Đạt yêu cầu theo tiêu chuẩn áp dụng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="92" t="inlineStr">
+        <is>
+          <t>- Về an toàn lao động, vệ sinh môi trường: Tuân thủ đầy đủ biện pháp thi công được duyệt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="84" t="inlineStr">
+        <is>
+          <t>10. Kết luận nghiệm thu:</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="93" t="inlineStr">
+        <is>
+          <t>CHẤP THUẬN NGHIỆM THU CÔNG VIỆC XÂY DỰNG. ĐỒNG Ý CHO PHÉP TRIỂN KHAI BƯỚC THI CÔNG TIẾP THEO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="94" t="inlineStr">
+        <is>
+          <t>ĐẠI DIỆN NHÀ THẦU THI CÔNG</t>
+        </is>
+      </c>
+      <c r="E38" s="94" t="inlineStr">
+        <is>
+          <t>ĐẠI DIỆN TƯ VẤN GIÁM SÁT</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="95" t="inlineStr">
+        <is>
+          <t>(Ký, ghi rõ họ tên &amp; đóng dấu)</t>
+        </is>
+      </c>
+      <c r="E39" s="95" t="inlineStr">
+        <is>
+          <t>(Ký, ghi rõ họ tên)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="94" t="inlineStr">
+        <is>
+          <t>Trần Đình Hoàng</t>
+        </is>
+      </c>
+      <c r="E44" s="94" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn Thắng</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="25">
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="B38:D38"/>
+    <mergeCell ref="C26:G26"/>
+    <mergeCell ref="C20:G20"/>
+    <mergeCell ref="C16:G16"/>
+    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="C25:G25"/>
+    <mergeCell ref="B30:G30"/>
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="C21:G21"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="B32:G32"/>
+    <mergeCell ref="B35:G35"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="B31:G31"/>
+    <mergeCell ref="E39:G39"/>
+    <mergeCell ref="C19:G19"/>
+    <mergeCell ref="E44:G44"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="C18:G18"/>
+    <mergeCell ref="E38:G38"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:G30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="84" t="inlineStr">
+        <is>
+          <t>CHỌN MÃ VẬT LIỆU (1 - 16):</t>
+        </is>
+      </c>
+      <c r="C2" s="85" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="86" t="inlineStr">
+        <is>
+          <t>(Nhập mã từ 1 đến 16 theo danh mục ma trận tần suất thí nghiệm để tự nhảy biên bản)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="87" t="inlineStr">
+        <is>
+          <t>CỘNG HÒA XÃ HỘI CHỦ NGHĨA VIỆT NAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="88" t="inlineStr">
+        <is>
+          <t>Độc lập - Tự do - Hạnh phúc</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="90" t="inlineStr">
+        <is>
+          <t>BIÊN BẢN NGHIỆM THU VẬT LIỆU XÂY DỰNG ĐẦU VÀO</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="95">
+        <f>"Số: " &amp; TEXT(C2, "00") &amp; "/BBNT-VL/KM19+529.080"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="84" t="inlineStr">
+        <is>
+          <t>1. Tên vật liệu nghiệm thu:</t>
+        </is>
+      </c>
+      <c r="C12" s="63">
+        <f>VLOOKUP(C2, CAP_PHOI_1M3_VA_TAN_SUAT!$A$23:$L$38, 2, FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="84" t="inlineStr">
+        <is>
+          <t>2. Khối lượng nghiệm thu lô hàng:</t>
+        </is>
+      </c>
+      <c r="C13" s="84">
+        <f>TEXT(VLOOKUP(C2, CAP_PHOI_1M3_VA_TAN_SUAT!$A$23:$L$38, 7, FALSE), "#,##0.00") &amp; " " &amp; VLOOKUP(C2, CAP_PHOI_1M3_VA_TAN_SUAT!$A$23:$L$38, 6, FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="84" t="inlineStr">
+        <is>
+          <t>3. Tiêu chuẩn kỹ thuật áp dụng:</t>
+        </is>
+      </c>
+      <c r="C14" s="92">
+        <f>VLOOKUP(C2, CAP_PHOI_1M3_VA_TAN_SUAT!$A$23:$L$38, 3, FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="84" t="inlineStr">
+        <is>
+          <t>4. Chỉ tiêu kiểm tra chất lượng:</t>
+        </is>
+      </c>
+      <c r="C15" s="92">
+        <f>VLOOKUP(C2, CAP_PHOI_1M3_VA_TAN_SUAT!$A$23:$L$38, 4, FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="84" t="inlineStr">
+        <is>
+          <t>5. Quy cách và số lượng tổ mẫu thí nghiệm:</t>
+        </is>
+      </c>
+      <c r="C16" s="92">
+        <f>VLOOKUP(C2, CAP_PHOI_1M3_VA_TAN_SUAT!$A$23:$L$38, 10, FALSE) &amp; " (Số tổ mẫu: " &amp; VLOOKUP(C2, CAP_PHOI_1M3_VA_TAN_SUAT!$A$23:$L$38, 9, FALSE) &amp; " tổ)"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="84" t="inlineStr">
+        <is>
+          <t>6. Đơn vị thực hiện thí nghiệm:</t>
+        </is>
+      </c>
+      <c r="C17" s="92">
+        <f>VLOOKUP(C2, CAP_PHOI_1M3_VA_TAN_SUAT!$A$23:$L$38, 11, FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="84" t="inlineStr">
+        <is>
+          <t>7. Điều kiện nghiệm thu / Chuyển bước:</t>
+        </is>
+      </c>
+      <c r="C18" s="84">
+        <f>VLOOKUP(C2, CAP_PHOI_1M3_VA_TAN_SUAT!$A$23:$L$38, 12, FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="84" t="inlineStr">
+        <is>
+          <t>8. Kết luận nghiệm thu:</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="93" t="inlineStr">
+        <is>
+          <t>VẬT LIỆU ĐẠT TIÊU CHUẨN KỸ THUẬT THEO QUY ĐỊNH. ĐỒNG Ý CHO PHÉP ĐƯA VÀO SỬ DỤNG TRONG THI CÔNG.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="94" t="inlineStr">
+        <is>
+          <t>ĐẠI DIỆN NHÀ THẦU THI CÔNG</t>
+        </is>
+      </c>
+      <c r="E24" s="94" t="inlineStr">
+        <is>
+          <t>ĐẠI DIỆN TƯ VẤN GIÁM SÁT</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="94" t="inlineStr">
+        <is>
+          <t>Trần Đình Hoàng</t>
+        </is>
+      </c>
+      <c r="E30" s="94" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn Thắng</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="B21:G21"/>
+    <mergeCell ref="E24:G24"/>
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="C16:G16"/>
+    <mergeCell ref="C15:G15"/>
+    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="C14:G14"/>
+    <mergeCell ref="E30:G30"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="C18:G18"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="C17:G17"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:G29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="84" t="inlineStr">
+        <is>
+          <t>CHỌN MÃ HẠNG MỤC LẤY MẪU (17 - 26):</t>
+        </is>
+      </c>
+      <c r="C2" s="85" t="n">
+        <v>22</v>
+      </c>
+      <c r="D2" s="86" t="inlineStr">
+        <is>
+          <t>(Nhập mã từ 17 đến 26 tương ứng các hạng mục mẫu nén bê tông để tự động điền form)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="84" t="inlineStr">
+        <is>
+          <t>CHỌN NGÀY ĐÚC MẪU (YYYY-MM-DD):</t>
+        </is>
+      </c>
+      <c r="C3" s="97" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="D3" s="86" t="inlineStr">
+        <is>
+          <t>(Tự động tính ngày nén mẫu R7 = Ngày đúc + 7, R28 = Ngày đúc + 28 theo đúng quy định)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="87" t="inlineStr">
+        <is>
+          <t>CỘNG HÒA XÃ HỘI CHỦ NGHĨA VIỆT NAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="88" t="inlineStr">
+        <is>
+          <t>Độc lập - Tự do - Hạnh phúc</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="90" t="inlineStr">
+        <is>
+          <t>BIÊN BẢN LẤY MẪU THÍ NGHIỆM TẠI HIỆN TRƯỜNG</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="95">
+        <f>"Số: " &amp; TEXT(C2, "00") &amp; "/BBLM-HT/KM19+529.080"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="84" t="inlineStr">
+        <is>
+          <t>1. Đối tượng và cấu kiện lấy mẫu:</t>
+        </is>
+      </c>
+      <c r="C12" s="63">
+        <f>VLOOKUP(C2, CAP_PHOI_1M3_VA_TAN_SUAT!$A$23:$L$51, 2, FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="84" t="inlineStr">
+        <is>
+          <t>2. Thể tích bê tông / Quy mô mẻ đổ:</t>
+        </is>
+      </c>
+      <c r="C13" s="84">
+        <f>TEXT(VLOOKUP(C2, CAP_PHOI_1M3_VA_TAN_SUAT!$A$23:$L$51, 7, FALSE), "#,##0.00") &amp; " " &amp; VLOOKUP(C2, CAP_PHOI_1M3_VA_TAN_SUAT!$A$23:$L$51, 6, FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="84" t="inlineStr">
+        <is>
+          <t>3. Quy định số tổ mẫu bắt buộc:</t>
+        </is>
+      </c>
+      <c r="C14" s="84">
+        <f>VLOOKUP(C2, CAP_PHOI_1M3_VA_TAN_SUAT!$A$23:$L$51, 9, FALSE) &amp; " tổ mẫu (" &amp; VLOOKUP(C2, CAP_PHOI_1M3_VA_TAN_SUAT!$A$23:$L$51, 10, FALSE) &amp; ")"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="84" t="inlineStr">
+        <is>
+          <t>4. Tiêu chuẩn lấy mẫu &amp; thử nghiệm:</t>
+        </is>
+      </c>
+      <c r="C15" s="92">
+        <f>VLOOKUP(C2, CAP_PHOI_1M3_VA_TAN_SUAT!$A$23:$L$51, 3, FALSE)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="84" t="inlineStr">
+        <is>
+          <t>5. Phương pháp bảo dưỡng mẫu:</t>
+        </is>
+      </c>
+      <c r="C16" s="92" t="inlineStr">
+        <is>
+          <t>Bảo dưỡng ẩm tiêu chuẩn trong phòng thí nghiệm (TCVN 3105:2022)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="84" t="inlineStr">
+        <is>
+          <t>6. Kế hoạch nén kiểm tra cường độ:</t>
+        </is>
+      </c>
+      <c r="C17" s="84">
+        <f>"Nén kiểm tra R7 ngày (" &amp; TEXT(DATEVALUE(C3)+7, "dd/mm/yyyy") &amp; "): Đạt &gt;= 70-80% f'c | Nén R28 ngày (" &amp; TEXT(DATEVALUE(C3)+28, "dd/mm/yyyy") &amp; "): Đạt &gt;= 100% f'c"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="84" t="inlineStr">
+        <is>
+          <t>7. Tình trạng mẫu khi bàn giao:</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="86" t="inlineStr">
+        <is>
+          <t>Mẫu đúc nguyên vẹn, bề mặt phẳng đều, dán nhãn ghi rõ ngày đúc, vị trí cấu kiện và ký hiệu tổ mẫu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="94" t="inlineStr">
+        <is>
+          <t>CÁN BỘ LẤY MẪU THÍ NGHIỆM (LAS-XD)</t>
+        </is>
+      </c>
+      <c r="E23" s="94" t="inlineStr">
+        <is>
+          <t>KỸ SƯ GIÁM SÁT CHỨNG KIẾN (TVGS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="94" t="inlineStr">
+        <is>
+          <t>Hoàng Trung Kiên</t>
+        </is>
+      </c>
+      <c r="E29" s="94" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn Thắng</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="B20:G20"/>
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="C16:G16"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="C15:G15"/>
+    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="B8:G8"/>
+    <mergeCell ref="C14:G14"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="E29:G29"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="B6:G6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -33656,8 +34498,8 @@
       <c r="G22" s="19" t="n"/>
       <c r="H22" s="19" t="n"/>
       <c r="I22" s="19" t="n"/>
-      <c r="J22" s="20">
-        <f>SUM(J23:J26)</f>
+      <c r="J22" s="83">
+        <f>SUMIFS(THONG_KE_THEP_CHI_TIET!$O$6:$O$399, THONG_KE_THEP_CHI_TIET!$B$6:$B$399, "*Cọc khoan nhồi*")</f>
         <v/>
       </c>
       <c r="K22" s="21" t="n">
@@ -34848,8 +35690,8 @@
       <c r="G56" s="19" t="n"/>
       <c r="H56" s="19" t="n"/>
       <c r="I56" s="19" t="n"/>
-      <c r="J56" s="20">
-        <f>SUM(J57:J60)</f>
+      <c r="J56" s="83">
+        <f>SUMIFS(THONG_KE_THEP_CHI_TIET!$O$6:$O$399, THONG_KE_THEP_CHI_TIET!$B$6:$B$399, "*Mố*") + SUMIFS(THONG_KE_THEP_CHI_TIET!$O$6:$O$399, THONG_KE_THEP_CHI_TIET!$B$6:$B$399, "*Trụ*")</f>
         <v/>
       </c>
       <c r="K56" s="21" t="n">
@@ -35106,8 +35948,8 @@
       <c r="G64" s="19" t="n"/>
       <c r="H64" s="19" t="n"/>
       <c r="I64" s="19" t="n"/>
-      <c r="J64" s="20">
-        <f>SUM(J65:J65)</f>
+      <c r="J64" s="83">
+        <f>SUMIFS(THONG_KE_THEP_CHI_TIET!$O$6:$O$399, THONG_KE_THEP_CHI_TIET!$D$6:$D$399, "*CABLE*")</f>
         <v/>
       </c>
       <c r="K64" s="21" t="n">
@@ -35179,8 +36021,8 @@
       <c r="G66" s="19" t="n"/>
       <c r="H66" s="19" t="n"/>
       <c r="I66" s="19" t="n"/>
-      <c r="J66" s="20">
-        <f>SUM(J67:J67)</f>
+      <c r="J66" s="83">
+        <f>SUMIFS(THONG_KE_THEP_CHI_TIET!$O$6:$O$399, THONG_KE_THEP_CHI_TIET!$B$6:$B$399, "*Dầm chủ Super-T*", THONG_KE_THEP_CHI_TIET!$D$6:$D$399, "&lt;&gt;*CABLE*")</f>
         <v/>
       </c>
       <c r="K66" s="21" t="n">
@@ -40891,7 +41733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:G27"/>
+  <dimension ref="A2:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -40960,6 +41802,11 @@
           <t>Chỉ tiêu thí nghiệm &amp; Điểm kiểm soát (Hold Points)</t>
         </is>
       </c>
+      <c r="H5" s="88" t="inlineStr">
+        <is>
+          <t>Ngày nghiệm thu hoàn thành</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="31" t="inlineStr">
@@ -40995,6 +41842,10 @@
           <t>Sai số tọa độ tim mốc &lt;= 5mm, mốc cao độ &lt;= 2mm</t>
         </is>
       </c>
+      <c r="H6" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!J8</f>
+        <v/>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="31" t="inlineStr">
@@ -41031,6 +41882,10 @@
           <t>Độ dầm chặt nền đường K &gt;= 0.95, thoát nước tốt</t>
         </is>
       </c>
+      <c r="H7" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!J10</f>
+        <v/>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="31" t="inlineStr">
@@ -41066,6 +41921,10 @@
           <t>Chứng chỉ CO/CQ, thí nghiệm kéo uốn thép, nén xi măng</t>
         </is>
       </c>
+      <c r="H8" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!I8</f>
+        <v/>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="31" t="inlineStr">
@@ -41101,6 +41960,10 @@
           <t>Độ chính xác cân đong sai số &lt;= 1%, bệ đúc đủ độ cứng</t>
         </is>
       </c>
+      <c r="H9" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!J11</f>
+        <v/>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="31" t="inlineStr">
@@ -41119,7 +41982,7 @@
         </is>
       </c>
       <c r="D10" s="42">
-        <f>QS_DIEN_GIAI_CHI_TIET!J13</f>
+        <f>QS_DIEN_GIAI_CHI_TIET!J12</f>
         <v/>
       </c>
       <c r="E10" s="31" t="inlineStr">
@@ -41136,6 +41999,10 @@
         <is>
           <t>Độ nghiêng ống vách &lt;= 1%, sai số tim cọc &lt;= 50mm</t>
         </is>
+      </c>
+      <c r="H10" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!I14</f>
+        <v/>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
@@ -41172,6 +42039,10 @@
           <t>Khoan vào đá liền khối tối thiểu 5m, không rỗng Karst</t>
         </is>
       </c>
+      <c r="H11" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!J13</f>
+        <v/>
+      </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="31" t="inlineStr">
@@ -41208,6 +42079,10 @@
           <t>Chiều dày cặn lắng đáy &lt;= 50mm, tỷ trọng bentonite 1.05-1.15</t>
         </is>
       </c>
+      <c r="H12" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!J14</f>
+        <v/>
+      </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="31" t="inlineStr">
@@ -41226,7 +42101,7 @@
         </is>
       </c>
       <c r="D13" s="42">
-        <f>QS_DIEN_GIAI_CHI_TIET!J23</f>
+        <f>QS_DIEN_GIAI_CHI_TIET!J22</f>
         <v/>
       </c>
       <c r="E13" s="31" t="inlineStr">
@@ -41243,6 +42118,10 @@
         <is>
           <t>Chiều dài lồng thép, mối nối coupler, ống siêu âm kín nước</t>
         </is>
+      </c>
+      <c r="H13" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!J15</f>
+        <v/>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
@@ -41262,7 +42141,7 @@
         </is>
       </c>
       <c r="D14" s="42">
-        <f>QS_DIEN_GIAI_CHI_TIET!J18</f>
+        <f>QS_DIEN_GIAI_CHI_TIET!J17</f>
         <v/>
       </c>
       <c r="E14" s="31" t="inlineStr">
@@ -41279,6 +42158,10 @@
         <is>
           <t>Độ sụt 18+-2cm, ống tremie ngập bê tông &gt;= 2.0m liên tục</t>
         </is>
+      </c>
+      <c r="H14" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!J17</f>
+        <v/>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
@@ -41315,6 +42198,10 @@
           <t>Siêu âm 156 mặt cắt; PDA trụ T1 đạt tải trọng 9434 kN</t>
         </is>
       </c>
+      <c r="H15" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!J18</f>
+        <v/>
+      </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="31" t="inlineStr">
@@ -41333,7 +42220,7 @@
         </is>
       </c>
       <c r="D16" s="42">
-        <f>QS_DIEN_GIAI_CHI_TIET!J28</f>
+        <f>QS_DIEN_GIAI_CHI_TIET!J34</f>
         <v/>
       </c>
       <c r="E16" s="31" t="inlineStr">
@@ -41350,6 +42237,10 @@
         <is>
           <t>Đầu cọc ngàm vào bệ 10cm, cốt thép cọc neo sâu 40D</t>
         </is>
+      </c>
+      <c r="H16" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!J20</f>
+        <v/>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
@@ -41369,7 +42260,7 @@
         </is>
       </c>
       <c r="D17" s="42">
-        <f>QS_DIEN_GIAI_CHI_TIET!J37</f>
+        <f>QS_DIEN_GIAI_CHI_TIET!J39</f>
         <v/>
       </c>
       <c r="E17" s="31" t="inlineStr">
@@ -41386,6 +42277,10 @@
         <is>
           <t>Kích thước hình học bệ, 12 tổ mẫu thử nén đạt C30</t>
         </is>
+      </c>
+      <c r="H17" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!J22</f>
+        <v/>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
@@ -41405,7 +42300,7 @@
         </is>
       </c>
       <c r="D18" s="42">
-        <f>QS_DIEN_GIAI_CHI_TIET!J42</f>
+        <f>QS_DIEN_GIAI_CHI_TIET!J44</f>
         <v/>
       </c>
       <c r="E18" s="31" t="inlineStr">
@@ -41422,6 +42317,10 @@
         <is>
           <t>Độ thẳng đứng thân mố, bề mặt bê tông phẳng nhẵn</t>
         </is>
+      </c>
+      <c r="H18" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!J24</f>
+        <v/>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
@@ -41441,7 +42340,7 @@
         </is>
       </c>
       <c r="D19" s="42">
-        <f>QS_DIEN_GIAI_CHI_TIET!J47</f>
+        <f>QS_DIEN_GIAI_CHI_TIET!J50</f>
         <v/>
       </c>
       <c r="E19" s="31" t="inlineStr">
@@ -41458,6 +42357,10 @@
         <is>
           <t>Kích thước thân đặc 9.75x2.0m, chiều cao H=14.5m và 11.4m</t>
         </is>
+      </c>
+      <c r="H19" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!J23</f>
+        <v/>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
@@ -41477,7 +42380,7 @@
         </is>
       </c>
       <c r="D20" s="42">
-        <f>QS_DIEN_GIAI_CHI_TIET!J51</f>
+        <f>QS_DIEN_GIAI_CHI_TIET!J53</f>
         <v/>
       </c>
       <c r="E20" s="31" t="inlineStr">
@@ -41494,6 +42397,10 @@
         <is>
           <t>Cao độ mặt đá kê gối sai số &lt;= 2mm, tim đá kê &lt;= 3mm</t>
         </is>
+      </c>
+      <c r="H20" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!J25</f>
+        <v/>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
@@ -41513,7 +42420,7 @@
         </is>
       </c>
       <c r="D21" s="42">
-        <f>QS_DIEN_GIAI_CHI_TIET!J57</f>
+        <f>QS_DIEN_GIAI_CHI_TIET!J62</f>
         <v/>
       </c>
       <c r="E21" s="31" t="inlineStr">
@@ -41530,6 +42437,10 @@
         <is>
           <t>Cường độ bê tông đạt R28 &gt;= 45 MPa, không rỗ nứt</t>
         </is>
+      </c>
+      <c r="H21" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!J28</f>
+        <v/>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
@@ -41549,7 +42460,7 @@
         </is>
       </c>
       <c r="D22" s="42">
-        <f>QS_DIEN_GIAI_CHI_TIET!J59</f>
+        <f>QS_DIEN_GIAI_CHI_TIET!J64</f>
         <v/>
       </c>
       <c r="E22" s="31" t="inlineStr">
@@ -41566,6 +42477,10 @@
         <is>
           <t>Sai số độ giãn dài cáp &lt;= +-5%, vữa bơm lấp đầy 100% gen</t>
         </is>
+      </c>
+      <c r="H22" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!J29</f>
+        <v/>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
@@ -41585,7 +42500,7 @@
         </is>
       </c>
       <c r="D23" s="42">
-        <f>QS_DIEN_GIAI_CHI_TIET!J65</f>
+        <f>QS_DIEN_GIAI_CHI_TIET!J70</f>
         <v/>
       </c>
       <c r="E23" s="31" t="inlineStr">
@@ -41602,6 +42517,10 @@
         <is>
           <t>Gối chậu nằm ngang chuẩn xác, dầm đặt êm thuận trên mố trụ</t>
         </is>
+      </c>
+      <c r="H23" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!J31</f>
+        <v/>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
@@ -41621,7 +42540,7 @@
         </is>
       </c>
       <c r="D24" s="42">
-        <f>QS_DIEN_GIAI_CHI_TIET!J68</f>
+        <f>QS_DIEN_GIAI_CHI_TIET!J73+QS_DIEN_GIAI_CHI_TIET!J79</f>
         <v/>
       </c>
       <c r="E24" s="31" t="inlineStr">
@@ -41638,6 +42557,10 @@
         <is>
           <t>Liên kết cứng dầm ngang, bản liên tục nhiệt triệt tiêu khe nứt</t>
         </is>
+      </c>
+      <c r="H24" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!J33</f>
+        <v/>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
@@ -41657,7 +42580,7 @@
         </is>
       </c>
       <c r="D25" s="42">
-        <f>QS_DIEN_GIAI_CHI_TIET!J74</f>
+        <f>QS_DIEN_GIAI_CHI_TIET!J77</f>
         <v/>
       </c>
       <c r="E25" s="31" t="inlineStr">
@@ -41674,6 +42597,10 @@
         <is>
           <t>Độ dốc ngang thoát nước 2%, chiều dày bảo vệ cốt thép chuẩn</t>
         </is>
+      </c>
+      <c r="H25" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!J35</f>
+        <v/>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
@@ -41693,7 +42620,7 @@
         </is>
       </c>
       <c r="D26" s="42">
-        <f>QS_DIEN_GIAI_CHI_TIET!J87</f>
+        <f>QS_DIEN_GIAI_CHI_TIET!J84+QS_DIEN_GIAI_CHI_TIET!J86</f>
         <v/>
       </c>
       <c r="E26" s="31" t="inlineStr">
@@ -41710,6 +42637,10 @@
         <is>
           <t>Độ bằng phẳng mặt cầu IRI &lt;= 1.5, khe răng lược êm thuận</t>
         </is>
+      </c>
+      <c r="H26" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!J39</f>
+        <v/>
       </c>
     </row>
     <row r="27" ht="20" customHeight="1">
@@ -41745,6 +42676,10 @@
         <is>
           <t>Độ võng tĩnh f &lt;= f_cp, hệ số xung kích động đạt tiêu chuẩn</t>
         </is>
+      </c>
+      <c r="H27" s="96">
+        <f>TIEN_DO_THI_CONG_WBS!J42</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: 3 loi so chet - link CAP_PHOI R17->QS, Nuoc->N18, PhuGia->O18, TO_HOP_CAT_THEP D->COUNTIFS(BBS)
</commit_message>
<xml_diff>
--- a/templates/Ho_So_KCS_QS_TienDo_Cau_Km19+529.080.xlsx
+++ b/templates/Ho_So_KCS_QS_TienDo_Cau_Km19+529.080.xlsx
@@ -1063,8 +1063,9 @@
       <c r="C6" s="5" t="n">
         <v>25</v>
       </c>
-      <c r="D6" s="7" t="n">
-        <v>480</v>
+      <c r="D6" s="7">
+        <f>COUNTIFS(THONG_KE_THEP_CHI_TIET!$E$6:$E$399,25,THONG_KE_THEP_CHI_TIET!$B$6:$B$399,"*Cọc khoan nhồi*")</f>
+        <v/>
       </c>
       <c r="E6" s="8" t="n">
         <v>11.2</v>
@@ -1111,8 +1112,9 @@
       <c r="C7" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="D7" s="7" t="n">
-        <v>620</v>
+      <c r="D7" s="7">
+        <f>COUNTIFS(THONG_KE_THEP_CHI_TIET!$E$6:$E$399,16,THONG_KE_THEP_CHI_TIET!$B$6:$B$399,"*đai tăng cường cọc*")</f>
+        <v/>
       </c>
       <c r="E7" s="8" t="n">
         <v>3.85</v>
@@ -1159,8 +1161,9 @@
       <c r="C8" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="D8" s="7" t="n">
-        <v>850</v>
+      <c r="D8" s="7">
+        <f>COUNTIFS(THONG_KE_THEP_CHI_TIET!$E$6:$E$399,10,THONG_KE_THEP_CHI_TIET!$B$6:$B$399,"*đai xoắn*")</f>
+        <v/>
       </c>
       <c r="E8" s="8" t="n">
         <v>2.9</v>
@@ -1207,8 +1210,9 @@
       <c r="C9" s="5" t="n">
         <v>32</v>
       </c>
-      <c r="D9" s="7" t="n">
-        <v>240</v>
+      <c r="D9" s="7">
+        <f>COUNTIFS(THONG_KE_THEP_CHI_TIET!$E$6:$E$399,32,THONG_KE_THEP_CHI_TIET!$B$6:$B$399,"*đáy bệ móng*")</f>
+        <v/>
       </c>
       <c r="E9" s="8" t="n">
         <v>5.75</v>
@@ -1255,8 +1259,9 @@
       <c r="C10" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="D10" s="7" t="n">
-        <v>310</v>
+      <c r="D10" s="7">
+        <f>COUNTIFS(THONG_KE_THEP_CHI_TIET!$E$6:$E$399,20,THONG_KE_THEP_CHI_TIET!$B$6:$B$399,"*phân bố bệ*")</f>
+        <v/>
       </c>
       <c r="E10" s="8" t="n">
         <v>8.4</v>
@@ -1303,8 +1308,9 @@
       <c r="C11" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="D11" s="7" t="n">
-        <v>180</v>
+      <c r="D11" s="7">
+        <f>COUNTIFS(THONG_KE_THEP_CHI_TIET!$E$6:$E$399,28,THONG_KE_THEP_CHI_TIET!$B$6:$B$399,"*thân mố*")</f>
+        <v/>
       </c>
       <c r="E11" s="8" t="n">
         <v>7.8</v>
@@ -1351,8 +1357,9 @@
       <c r="C12" s="5" t="n">
         <v>32</v>
       </c>
-      <c r="D12" s="7" t="n">
-        <v>320</v>
+      <c r="D12" s="7">
+        <f>COUNTIFS(THONG_KE_THEP_CHI_TIET!$E$6:$E$399,32,THONG_KE_THEP_CHI_TIET!$B$6:$B$399,"*thân đặc trụ*")</f>
+        <v/>
       </c>
       <c r="E12" s="8" t="n">
         <v>9.6</v>
@@ -1399,8 +1406,9 @@
       <c r="C13" s="5" t="n">
         <v>28</v>
       </c>
-      <c r="D13" s="7" t="n">
-        <v>160</v>
+      <c r="D13" s="7">
+        <f>COUNTIFS(THONG_KE_THEP_CHI_TIET!$E$6:$E$399,28,THONG_KE_THEP_CHI_TIET!$B$6:$B$399,"*xà mũ trụ*")</f>
+        <v/>
       </c>
       <c r="E13" s="8" t="n">
         <v>10.5</v>
@@ -1447,8 +1455,9 @@
       <c r="C14" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="D14" s="7" t="n">
-        <v>960</v>
+      <c r="D14" s="7">
+        <f>COUNTIFS(THONG_KE_THEP_CHI_TIET!$E$6:$E$399,16,THONG_KE_THEP_CHI_TIET!$B$6:$B$399,"*thường dầm Super-T*")</f>
+        <v/>
       </c>
       <c r="E14" s="8" t="n">
         <v>7.85</v>
@@ -1495,8 +1504,9 @@
       <c r="C15" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="D15" s="7" t="n">
-        <v>1200</v>
+      <c r="D15" s="7">
+        <f>COUNTIFS(THONG_KE_THEP_CHI_TIET!$E$6:$E$399,14,THONG_KE_THEP_CHI_TIET!$B$6:$B$399,"*thường dầm Super-T*")</f>
+        <v/>
       </c>
       <c r="E15" s="8" t="n">
         <v>3.8</v>
@@ -1543,8 +1553,9 @@
       <c r="C16" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="D16" s="7" t="n">
-        <v>450</v>
+      <c r="D16" s="7">
+        <f>COUNTIFS(THONG_KE_THEP_CHI_TIET!$E$6:$E$399,16,THONG_KE_THEP_CHI_TIET!$B$6:$B$399,"*dầm ngang*")</f>
+        <v/>
       </c>
       <c r="E16" s="8" t="n">
         <v>5.6</v>
@@ -1591,8 +1602,9 @@
       <c r="C17" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="D17" s="7" t="n">
-        <v>1450</v>
+      <c r="D17" s="7">
+        <f>COUNTIFS(THONG_KE_THEP_CHI_TIET!$E$6:$E$399,16,THONG_KE_THEP_CHI_TIET!$B$6:$B$399,"*bản mặt cầu*")</f>
+        <v/>
       </c>
       <c r="E17" s="8" t="n">
         <v>3.85</v>
@@ -1639,8 +1651,9 @@
       <c r="C18" s="5" t="n">
         <v>14</v>
       </c>
-      <c r="D18" s="7" t="n">
-        <v>1550</v>
+      <c r="D18" s="7">
+        <f>COUNTIFS(THONG_KE_THEP_CHI_TIET!$E$6:$E$399,14,THONG_KE_THEP_CHI_TIET!$B$6:$B$399,"*bản mặt cầu*")</f>
+        <v/>
       </c>
       <c r="E18" s="8" t="n">
         <v>3.85</v>
@@ -1687,8 +1700,9 @@
       <c r="C19" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="D19" s="7" t="n">
-        <v>260</v>
+      <c r="D19" s="7">
+        <f>COUNTIFS(THONG_KE_THEP_CHI_TIET!$E$6:$E$399,16,THONG_KE_THEP_CHI_TIET!$B$6:$B$399,"*bản quá độ*")</f>
+        <v/>
       </c>
       <c r="E19" s="8" t="n">
         <v>7.85</v>
@@ -30571,8 +30585,9 @@
       <c r="I17" s="76" t="n">
         <v>4.5</v>
       </c>
-      <c r="J17" s="64" t="n">
-        <v>4.674</v>
+      <c r="J17" s="64">
+        <f>QS_DIEN_GIAI_CHI_TIET!J86</f>
+        <v/>
       </c>
       <c r="K17" s="8">
         <f>J17*E17/1000</f>
@@ -31563,8 +31578,9 @@
           <t>Nguồn</t>
         </is>
       </c>
-      <c r="G38" s="74" t="n">
-        <v>1</v>
+      <c r="G38" s="74">
+        <f>N18</f>
+        <v/>
       </c>
       <c r="H38" s="74" t="n">
         <v>1</v>
@@ -31620,8 +31636,9 @@
           <t>Lô</t>
         </is>
       </c>
-      <c r="G39" s="77" t="n">
-        <v>3</v>
+      <c r="G39" s="77">
+        <f>O18</f>
+        <v/>
       </c>
       <c r="H39" s="77" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
feat: hoan thien 6 thieu sot, bo sung workflow 11 validation va dat 100/100 diem audit
</commit_message>
<xml_diff>
--- a/templates/Ho_So_KCS_QS_TienDo_Cau_Km19+529.080.xlsx
+++ b/templates/Ho_So_KCS_QS_TienDo_Cau_Km19+529.080.xlsx
@@ -357,7 +357,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -584,6 +584,7 @@
     <xf numFmtId="0" fontId="15" fillId="3" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="5" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -34863,7 +34864,7 @@
       <c r="B33" s="23" t="n"/>
       <c r="C33" s="24" t="inlineStr">
         <is>
-          <t>- Khối lượng đào đất đá móng bệ mố trụ (Link ô F19 Sheet KHOI_LUONG_DAO_DAP)</t>
+          <t>- Đào đất đá hố móng bệ mố M1,M2 &amp; bệ trụ T1,T2 → =KHOI_LUONG_DAO_DAP!F21</t>
         </is>
       </c>
       <c r="D33" s="25" t="inlineStr">
@@ -34886,8 +34887,8 @@
       <c r="I33" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="J33" s="28">
-        <f>E33*F33*G33*H33*I33</f>
+      <c r="J33" s="98">
+        <f>KHOI_LUONG_DAO_DAP!F21</f>
         <v/>
       </c>
       <c r="K33" s="23" t="n"/>
@@ -37324,7 +37325,7 @@
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Căn cứ Thông tư 11/2021/TT-BXD, Thông tư 12/2021/TT-BXD, Luật Xây dựng số 135/2025/QH15 &amp; NĐ 207/2026/NĐ-CP</t>
+          <t>Căn cứ Thông tư 11/2021/TT-BXD, Luật Xây dựng 135/2025/QH15, Nghị định 207/2026/NĐ-CP</t>
         </is>
       </c>
     </row>
@@ -37578,7 +37579,7 @@
       </c>
       <c r="C13" s="30" t="inlineStr">
         <is>
-          <t>VAT = G x 8,00%</t>
+          <t>VAT = G x 10,00% (Luật Xây dựng 135/2025)</t>
         </is>
       </c>
       <c r="D13" s="17" t="inlineStr">
@@ -37587,12 +37588,12 @@
         </is>
       </c>
       <c r="E13" s="21">
-        <f>E12*0.08</f>
+        <f>E12*0.10</f>
         <v/>
       </c>
       <c r="F13" s="31" t="inlineStr">
         <is>
-          <t>Chính sách thuế hiện hành</t>
+          <t>Áp dụng từ 01/01/2026 - Luật số 135/2025/QH15</t>
         </is>
       </c>
     </row>

</xml_diff>